<commit_message>
add new mode: now clubs are from Champions League update data source file add new logos
</commit_message>
<xml_diff>
--- a/DataForSpatialGame.xlsx
+++ b/DataForSpatialGame.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ксюшенька\PycharmProjects\py-game-spatial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B647085-0627-4051-8C53-851AD56249B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98811EA-A438-4B06-9F54-94B4FA527B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13416" yWindow="1332" windowWidth="10836" windowHeight="11148" xr2:uid="{AEB23EE1-9EC4-42C4-A600-9555917A228B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{AEB23EE1-9EC4-42C4-A600-9555917A228B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="England" sheetId="1" r:id="rId1"/>
+    <sheet name="Champions League" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="180">
   <si>
     <t>club</t>
   </si>
@@ -262,6 +263,309 @@
   </si>
   <si>
     <t>Fratton Park</t>
+  </si>
+  <si>
+    <t>Real Madrid</t>
+  </si>
+  <si>
+    <t>Barcelona</t>
+  </si>
+  <si>
+    <t>Bayern Munich</t>
+  </si>
+  <si>
+    <t>Santiago Bernabéu</t>
+  </si>
+  <si>
+    <t>Madrid</t>
+  </si>
+  <si>
+    <t>40.4531</t>
+  </si>
+  <si>
+    <t>-3.6883</t>
+  </si>
+  <si>
+    <t>Camp Nou</t>
+  </si>
+  <si>
+    <t>41.3809</t>
+  </si>
+  <si>
+    <t>2.1228</t>
+  </si>
+  <si>
+    <t>Atletico Madrid</t>
+  </si>
+  <si>
+    <t>Cívitas Metropolitano</t>
+  </si>
+  <si>
+    <t>40.4362</t>
+  </si>
+  <si>
+    <t>-3.5995</t>
+  </si>
+  <si>
+    <t>53.4831</t>
+  </si>
+  <si>
+    <t>-2.2004</t>
+  </si>
+  <si>
+    <t>Emirates Stadium</t>
+  </si>
+  <si>
+    <t>51.5549</t>
+  </si>
+  <si>
+    <t>-0.1084</t>
+  </si>
+  <si>
+    <t>53.4308</t>
+  </si>
+  <si>
+    <t>-2.9608</t>
+  </si>
+  <si>
+    <t>Allianz Arena</t>
+  </si>
+  <si>
+    <t>Munich</t>
+  </si>
+  <si>
+    <t>48.2188</t>
+  </si>
+  <si>
+    <t>Borussia Dortmund</t>
+  </si>
+  <si>
+    <t>Signal Iduna Park</t>
+  </si>
+  <si>
+    <t>Dortmund</t>
+  </si>
+  <si>
+    <t>51.4926</t>
+  </si>
+  <si>
+    <t>Bayer Leverkusen</t>
+  </si>
+  <si>
+    <t>BayArena</t>
+  </si>
+  <si>
+    <t>Leverkusen</t>
+  </si>
+  <si>
+    <t>51.0383</t>
+  </si>
+  <si>
+    <t>7.0022</t>
+  </si>
+  <si>
+    <t>Inter Milan</t>
+  </si>
+  <si>
+    <t>San Siro</t>
+  </si>
+  <si>
+    <t>Milan</t>
+  </si>
+  <si>
+    <t>45.4781</t>
+  </si>
+  <si>
+    <t>9.1240</t>
+  </si>
+  <si>
+    <t>Juventus</t>
+  </si>
+  <si>
+    <t>Allianz Stadium</t>
+  </si>
+  <si>
+    <t>Turin</t>
+  </si>
+  <si>
+    <t>45.0994</t>
+  </si>
+  <si>
+    <t>Atalanta</t>
+  </si>
+  <si>
+    <t>Gewiss Stadium</t>
+  </si>
+  <si>
+    <t>Bergamo</t>
+  </si>
+  <si>
+    <t>45.7092</t>
+  </si>
+  <si>
+    <t>Paris Saint-Germain</t>
+  </si>
+  <si>
+    <t>Parc des Princes</t>
+  </si>
+  <si>
+    <t>Paris</t>
+  </si>
+  <si>
+    <t>48.8414</t>
+  </si>
+  <si>
+    <t>Monaco</t>
+  </si>
+  <si>
+    <t>Stade Louis II</t>
+  </si>
+  <si>
+    <t>43.7276</t>
+  </si>
+  <si>
+    <t>Sporting CP</t>
+  </si>
+  <si>
+    <t>Estádio José Alvalade</t>
+  </si>
+  <si>
+    <t>Lisbon</t>
+  </si>
+  <si>
+    <t>38.7612</t>
+  </si>
+  <si>
+    <t>-9.1604</t>
+  </si>
+  <si>
+    <t>Benfica</t>
+  </si>
+  <si>
+    <t>Estádio da Luz</t>
+  </si>
+  <si>
+    <t>38.7528</t>
+  </si>
+  <si>
+    <t>-9.1847</t>
+  </si>
+  <si>
+    <t>PSV Eindhoven</t>
+  </si>
+  <si>
+    <t>Philips Stadion</t>
+  </si>
+  <si>
+    <t>Eindhoven</t>
+  </si>
+  <si>
+    <t>51.4417</t>
+  </si>
+  <si>
+    <t>Club Brugge</t>
+  </si>
+  <si>
+    <t>Jan Breydel Stadium</t>
+  </si>
+  <si>
+    <t>Bruges</t>
+  </si>
+  <si>
+    <t>Prague</t>
+  </si>
+  <si>
+    <t>Kairat</t>
+  </si>
+  <si>
+    <t>Central Stadium</t>
+  </si>
+  <si>
+    <t>Almaty</t>
+  </si>
+  <si>
+    <t>Napoli</t>
+  </si>
+  <si>
+    <t>Olympiacos</t>
+  </si>
+  <si>
+    <t>Stadio Diego Armando Maradona</t>
+  </si>
+  <si>
+    <t>Aspmyra Stadion</t>
+  </si>
+  <si>
+    <t>Karaiskakis Stadium</t>
+  </si>
+  <si>
+    <t>Naples</t>
+  </si>
+  <si>
+    <t>Bodø</t>
+  </si>
+  <si>
+    <t>Piraeus</t>
+  </si>
+  <si>
+    <t>Qarabag</t>
+  </si>
+  <si>
+    <t>Tofiq Bahramov Stadium</t>
+  </si>
+  <si>
+    <t>Baku</t>
+  </si>
+  <si>
+    <t>Pafos</t>
+  </si>
+  <si>
+    <t>Stelios Kyriakides Stadium</t>
+  </si>
+  <si>
+    <t>Paphos</t>
+  </si>
+  <si>
+    <t>Copenhagen</t>
+  </si>
+  <si>
+    <t>Parken Stadium</t>
+  </si>
+  <si>
+    <t>Deutsche Bank Park</t>
+  </si>
+  <si>
+    <t>Frankfurt</t>
+  </si>
+  <si>
+    <t>Ajax</t>
+  </si>
+  <si>
+    <t>Johan Cruyff Arena</t>
+  </si>
+  <si>
+    <t>Amsterdam</t>
+  </si>
+  <si>
+    <t>Galatasaray</t>
+  </si>
+  <si>
+    <t>Rams Park</t>
+  </si>
+  <si>
+    <t>Istanbul</t>
+  </si>
+  <si>
+    <t>Slavia Prague</t>
+  </si>
+  <si>
+    <t>Fortuna Arena</t>
+  </si>
+  <si>
+    <t>Eintracht Frankfurt</t>
+  </si>
+  <si>
+    <t>Bodø Glimt</t>
   </si>
 </sst>
 </file>
@@ -305,9 +609,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1180,4 +1485,547 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45D669C2-4D92-485E-AAE3-CDC409B4E1B4}">
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.44140625" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" customWidth="1"/>
+    <col min="4" max="5" width="10.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>160</v>
+      </c>
+      <c r="B5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5">
+        <v>40.39</v>
+      </c>
+      <c r="E5" s="2">
+        <v>49.878100000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9">
+        <v>51.481699999999996</v>
+      </c>
+      <c r="E9">
+        <v>-0.191</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" t="s">
+        <v>100</v>
+      </c>
+      <c r="C10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D10" t="s">
+        <v>102</v>
+      </c>
+      <c r="E10" s="2">
+        <v>11.624700000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="2">
+        <v>956753</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" t="s">
+        <v>108</v>
+      </c>
+      <c r="C12" t="s">
+        <v>109</v>
+      </c>
+      <c r="D12" t="s">
+        <v>110</v>
+      </c>
+      <c r="E12" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>145</v>
+      </c>
+      <c r="B13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D13">
+        <v>51.211500000000001</v>
+      </c>
+      <c r="E13" s="2">
+        <v>3.1808000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" t="s">
+        <v>165</v>
+      </c>
+      <c r="D14">
+        <v>34.761400000000002</v>
+      </c>
+      <c r="E14" s="2">
+        <v>32.435299999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>112</v>
+      </c>
+      <c r="B15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" t="s">
+        <v>114</v>
+      </c>
+      <c r="D15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>176</v>
+      </c>
+      <c r="B16" t="s">
+        <v>177</v>
+      </c>
+      <c r="C16" t="s">
+        <v>148</v>
+      </c>
+      <c r="D16">
+        <v>50.067500000000003</v>
+      </c>
+      <c r="E16">
+        <v>14.4717</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" t="s">
+        <v>118</v>
+      </c>
+      <c r="C17" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" t="s">
+        <v>120</v>
+      </c>
+      <c r="E17" s="2">
+        <v>7.6413000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" t="s">
+        <v>122</v>
+      </c>
+      <c r="C18" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" t="s">
+        <v>124</v>
+      </c>
+      <c r="E18" s="2">
+        <v>9.6807999999999996</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>166</v>
+      </c>
+      <c r="B19" t="s">
+        <v>167</v>
+      </c>
+      <c r="C19" t="s">
+        <v>166</v>
+      </c>
+      <c r="D19">
+        <v>55.702800000000003</v>
+      </c>
+      <c r="E19" s="2">
+        <v>12.5717</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>125</v>
+      </c>
+      <c r="B20" t="s">
+        <v>126</v>
+      </c>
+      <c r="C20" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" t="s">
+        <v>128</v>
+      </c>
+      <c r="E20" s="2">
+        <v>2.2530000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" t="s">
+        <v>130</v>
+      </c>
+      <c r="C21" t="s">
+        <v>129</v>
+      </c>
+      <c r="D21" t="s">
+        <v>131</v>
+      </c>
+      <c r="E21" s="2">
+        <v>7.4154999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>178</v>
+      </c>
+      <c r="B22" t="s">
+        <v>168</v>
+      </c>
+      <c r="C22" t="s">
+        <v>169</v>
+      </c>
+      <c r="D22">
+        <v>50.068600000000004</v>
+      </c>
+      <c r="E22">
+        <v>8.6454000000000004</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>170</v>
+      </c>
+      <c r="B23" t="s">
+        <v>171</v>
+      </c>
+      <c r="C23" t="s">
+        <v>172</v>
+      </c>
+      <c r="D23">
+        <v>52.314399999999999</v>
+      </c>
+      <c r="E23">
+        <v>4.9419000000000004</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>132</v>
+      </c>
+      <c r="B24" t="s">
+        <v>133</v>
+      </c>
+      <c r="C24" t="s">
+        <v>134</v>
+      </c>
+      <c r="D24" t="s">
+        <v>135</v>
+      </c>
+      <c r="E24" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>137</v>
+      </c>
+      <c r="B25" t="s">
+        <v>138</v>
+      </c>
+      <c r="C25" t="s">
+        <v>134</v>
+      </c>
+      <c r="D25" t="s">
+        <v>139</v>
+      </c>
+      <c r="E25" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26" t="s">
+        <v>143</v>
+      </c>
+      <c r="D26" t="s">
+        <v>144</v>
+      </c>
+      <c r="E26" s="2">
+        <v>5.4673999999999996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27" t="s">
+        <v>174</v>
+      </c>
+      <c r="C27" t="s">
+        <v>175</v>
+      </c>
+      <c r="D27">
+        <v>41.103400000000001</v>
+      </c>
+      <c r="E27" s="2">
+        <v>28.991</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>149</v>
+      </c>
+      <c r="B28" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" t="s">
+        <v>151</v>
+      </c>
+      <c r="D28">
+        <v>43.238300000000002</v>
+      </c>
+      <c r="E28">
+        <v>76.924199999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>152</v>
+      </c>
+      <c r="B29" t="s">
+        <v>154</v>
+      </c>
+      <c r="C29" t="s">
+        <v>157</v>
+      </c>
+      <c r="D29">
+        <v>40.8279</v>
+      </c>
+      <c r="E29">
+        <v>14.193</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30" t="s">
+        <v>155</v>
+      </c>
+      <c r="C30" t="s">
+        <v>158</v>
+      </c>
+      <c r="D30">
+        <v>67.276600000000002</v>
+      </c>
+      <c r="E30">
+        <v>14.3927</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>153</v>
+      </c>
+      <c r="B31" t="s">
+        <v>156</v>
+      </c>
+      <c r="C31" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31">
+        <v>37.946399999999997</v>
+      </c>
+      <c r="E31">
+        <v>23.664400000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add new mode: find country from player's image update data source file
</commit_message>
<xml_diff>
--- a/DataForSpatialGame.xlsx
+++ b/DataForSpatialGame.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ксюшенька\PycharmProjects\py-game-spatial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98811EA-A438-4B06-9F54-94B4FA527B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4FFB3E6-0EFD-49A2-8125-71D3938AE4AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{AEB23EE1-9EC4-42C4-A600-9555917A228B}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="1" activeTab="2" xr2:uid="{AEB23EE1-9EC4-42C4-A600-9555917A228B}"/>
   </bookViews>
   <sheets>
     <sheet name="England" sheetId="1" r:id="rId1"/>
     <sheet name="Champions League" sheetId="2" r:id="rId2"/>
+    <sheet name="Players" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="264">
   <si>
     <t>club</t>
   </si>
@@ -566,6 +567,258 @@
   </si>
   <si>
     <t>Bodø Glimt</t>
+  </si>
+  <si>
+    <t>player</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>Ousmane Dembele</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Lamine Yamal</t>
+  </si>
+  <si>
+    <t>Spain</t>
+  </si>
+  <si>
+    <t>Vitinha</t>
+  </si>
+  <si>
+    <t>Portugal</t>
+  </si>
+  <si>
+    <t>Kylian Mbappe</t>
+  </si>
+  <si>
+    <t>Cole Palmer</t>
+  </si>
+  <si>
+    <t>England</t>
+  </si>
+  <si>
+    <t>Gianluigi Donnarumma</t>
+  </si>
+  <si>
+    <t>Nuno Mendes</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Pedri</t>
+  </si>
+  <si>
+    <t>Khvicha Kvaratskhelia</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>Harry Kane</t>
+  </si>
+  <si>
+    <t>Desire Doue</t>
+  </si>
+  <si>
+    <t>Viktor Gyokeres</t>
+  </si>
+  <si>
+    <t>Sweden</t>
+  </si>
+  <si>
+    <t>Robert Lewandowski</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Scott McTominay</t>
+  </si>
+  <si>
+    <t>Joao Neves</t>
+  </si>
+  <si>
+    <t>Scotland</t>
+  </si>
+  <si>
+    <t>Jude Bellingham</t>
+  </si>
+  <si>
+    <t>Fabian Ruiz</t>
+  </si>
+  <si>
+    <t>Denzel Dumfries</t>
+  </si>
+  <si>
+    <t>Netherlands</t>
+  </si>
+  <si>
+    <t>Erling Haaland</t>
+  </si>
+  <si>
+    <t>Norway</t>
+  </si>
+  <si>
+    <t>Declan Rice</t>
+  </si>
+  <si>
+    <t>Virgil Van Dijk</t>
+  </si>
+  <si>
+    <t>Florian Wirtz</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>Michael Olise</t>
+  </si>
+  <si>
+    <t>Bukayo Saka</t>
+  </si>
+  <si>
+    <t>William Saliba</t>
+  </si>
+  <si>
+    <t>David Raya</t>
+  </si>
+  <si>
+    <t>Dominik Szoboszlai</t>
+  </si>
+  <si>
+    <t>Hungary</t>
+  </si>
+  <si>
+    <t>Luka Modric</t>
+  </si>
+  <si>
+    <t>Croatia</t>
+  </si>
+  <si>
+    <t>Granit Xhaka</t>
+  </si>
+  <si>
+    <t>Switzerland</t>
+  </si>
+  <si>
+    <t>Arda Guler</t>
+  </si>
+  <si>
+    <t>Turkey</t>
+  </si>
+  <si>
+    <t>Andriy Shevchenko</t>
+  </si>
+  <si>
+    <t>Ukraine</t>
+  </si>
+  <si>
+    <t>Thierry Henry</t>
+  </si>
+  <si>
+    <t>Pavel Nedved</t>
+  </si>
+  <si>
+    <t>Czech Republic</t>
+  </si>
+  <si>
+    <t>Wayne Rooney</t>
+  </si>
+  <si>
+    <t>Paolo Maldini</t>
+  </si>
+  <si>
+    <t>Zinedine Zidane</t>
+  </si>
+  <si>
+    <t>Raul</t>
+  </si>
+  <si>
+    <t>Oliver Kahn</t>
+  </si>
+  <si>
+    <t>Dennis Bergkamp</t>
+  </si>
+  <si>
+    <t>Michael Ballack</t>
+  </si>
+  <si>
+    <t>Alessandro Del Piero</t>
+  </si>
+  <si>
+    <t>Michael Owen</t>
+  </si>
+  <si>
+    <t>David Beckham</t>
+  </si>
+  <si>
+    <t>Francesco Totti</t>
+  </si>
+  <si>
+    <t>Luis Figo</t>
+  </si>
+  <si>
+    <t>Henrik Larsson</t>
+  </si>
+  <si>
+    <t>Alessandro Nesta</t>
+  </si>
+  <si>
+    <t>Zlatko Zahovic</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>Roy Keane</t>
+  </si>
+  <si>
+    <t>Republic of Ireland</t>
+  </si>
+  <si>
+    <t>Lothar Matthaus</t>
+  </si>
+  <si>
+    <t>Jaap Stam</t>
+  </si>
+  <si>
+    <t>Peter Schmeichel</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>Ryan Giggs</t>
+  </si>
+  <si>
+    <t>Wales</t>
+  </si>
+  <si>
+    <t>Davor Suker</t>
+  </si>
+  <si>
+    <t>Edgar Davids</t>
+  </si>
+  <si>
+    <t>Michael Laudrup</t>
+  </si>
+  <si>
+    <t>Marc Overmars</t>
+  </si>
+  <si>
+    <t>Patrick Vieira</t>
+  </si>
+  <si>
+    <t>Ruud van Nistelrooy</t>
+  </si>
+  <si>
+    <t>Lilian Thuram</t>
   </si>
 </sst>
 </file>
@@ -609,10 +862,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1579,7 +1831,7 @@
       <c r="D5">
         <v>40.39</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5">
         <v>49.878100000000003</v>
       </c>
     </row>
@@ -1664,7 +1916,7 @@
       <c r="D10" t="s">
         <v>102</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10">
         <v>11.624700000000001</v>
       </c>
     </row>
@@ -1681,8 +1933,8 @@
       <c r="D11" t="s">
         <v>106</v>
       </c>
-      <c r="E11" s="2">
-        <v>956753</v>
+      <c r="E11">
+        <v>7.4519000000000002</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -1715,7 +1967,7 @@
       <c r="D13">
         <v>51.211500000000001</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13">
         <v>3.1808000000000001</v>
       </c>
     </row>
@@ -1732,7 +1984,7 @@
       <c r="D14">
         <v>34.761400000000002</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14">
         <v>32.435299999999998</v>
       </c>
     </row>
@@ -1783,7 +2035,7 @@
       <c r="D17" t="s">
         <v>120</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17">
         <v>7.6413000000000002</v>
       </c>
     </row>
@@ -1800,7 +2052,7 @@
       <c r="D18" t="s">
         <v>124</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18">
         <v>9.6807999999999996</v>
       </c>
     </row>
@@ -1817,7 +2069,7 @@
       <c r="D19">
         <v>55.702800000000003</v>
       </c>
-      <c r="E19" s="2">
+      <c r="E19">
         <v>12.5717</v>
       </c>
     </row>
@@ -1834,7 +2086,7 @@
       <c r="D20" t="s">
         <v>128</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20">
         <v>2.2530000000000001</v>
       </c>
     </row>
@@ -1851,7 +2103,7 @@
       <c r="D21" t="s">
         <v>131</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21">
         <v>7.4154999999999998</v>
       </c>
     </row>
@@ -1936,7 +2188,7 @@
       <c r="D26" t="s">
         <v>144</v>
       </c>
-      <c r="E26" s="2">
+      <c r="E26">
         <v>5.4673999999999996</v>
       </c>
     </row>
@@ -1953,7 +2205,7 @@
       <c r="D27">
         <v>41.103400000000001</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27">
         <v>28.991</v>
       </c>
     </row>
@@ -2023,6 +2275,508 @@
       </c>
       <c r="E31">
         <v>23.664400000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{109B8CC7-D254-49D1-937A-38C4F2A22541}">
+  <dimension ref="A1:B61"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B7" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>192</v>
+      </c>
+      <c r="B8" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>194</v>
+      </c>
+      <c r="B9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B10" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>197</v>
+      </c>
+      <c r="B11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>198</v>
+      </c>
+      <c r="B12" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>199</v>
+      </c>
+      <c r="B13" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B14" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>203</v>
+      </c>
+      <c r="B15" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>204</v>
+      </c>
+      <c r="B16" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>206</v>
+      </c>
+      <c r="B17" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>207</v>
+      </c>
+      <c r="B18" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>208</v>
+      </c>
+      <c r="B19" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>212</v>
+      </c>
+      <c r="B21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>213</v>
+      </c>
+      <c r="B22" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>214</v>
+      </c>
+      <c r="B23" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>216</v>
+      </c>
+      <c r="B24" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>217</v>
+      </c>
+      <c r="B25" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>218</v>
+      </c>
+      <c r="B26" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>219</v>
+      </c>
+      <c r="B27" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>220</v>
+      </c>
+      <c r="B28" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>222</v>
+      </c>
+      <c r="B29" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>224</v>
+      </c>
+      <c r="B30" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>226</v>
+      </c>
+      <c r="B31" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>228</v>
+      </c>
+      <c r="B32" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>230</v>
+      </c>
+      <c r="B33" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>231</v>
+      </c>
+      <c r="B34" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>233</v>
+      </c>
+      <c r="B35" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>234</v>
+      </c>
+      <c r="B36" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>235</v>
+      </c>
+      <c r="B37" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>262</v>
+      </c>
+      <c r="B38" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>236</v>
+      </c>
+      <c r="B39" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>237</v>
+      </c>
+      <c r="B40" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>238</v>
+      </c>
+      <c r="B41" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>239</v>
+      </c>
+      <c r="B42" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>240</v>
+      </c>
+      <c r="B43" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>241</v>
+      </c>
+      <c r="B44" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>261</v>
+      </c>
+      <c r="B45" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>242</v>
+      </c>
+      <c r="B46" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>243</v>
+      </c>
+      <c r="B47" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>244</v>
+      </c>
+      <c r="B48" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>245</v>
+      </c>
+      <c r="B49" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>246</v>
+      </c>
+      <c r="B50" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>247</v>
+      </c>
+      <c r="B51" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>249</v>
+      </c>
+      <c r="B52" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>251</v>
+      </c>
+      <c r="B53" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>252</v>
+      </c>
+      <c r="B54" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>253</v>
+      </c>
+      <c r="B55" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>255</v>
+      </c>
+      <c r="B56" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>257</v>
+      </c>
+      <c r="B57" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>258</v>
+      </c>
+      <c r="B58" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>263</v>
+      </c>
+      <c r="B59" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>259</v>
+      </c>
+      <c r="B60" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>260</v>
+      </c>
+      <c r="B61" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>